<commit_message>
fix: marcador Tipo_plantilla como celda única oculta, no por fila
El control de tipo de plantilla (MATERIALES/CATEGORIAS) ahora solo se
escribe una vez (fila de encabezado + primera fila de dato) en vez de
repetirse en cada registro, y la columna queda oculta. La validación en
bulk-upload/bulk-validate no cambia: ya leía solo la primera fila.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/plantilla_materiales.xlsx
+++ b/templates/plantilla_materiales.xlsx
@@ -400,6 +400,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:K150"/>
+  <cols>
+    <col min="1" max="1"/>
+    <col min="2" max="2"/>
+    <col min="3" max="3"/>
+    <col min="4" max="4"/>
+    <col min="5" max="5"/>
+    <col min="6" max="6"/>
+    <col min="7" max="7"/>
+    <col min="8" max="8"/>
+    <col min="9" max="9"/>
+    <col min="10" max="10"/>
+    <col min="11" max="11" hidden="true"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -488,7 +501,7 @@
         <v/>
       </c>
       <c r="K3" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="4">
@@ -520,7 +533,7 @@
         <v/>
       </c>
       <c r="K4" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="5">
@@ -552,7 +565,7 @@
         <v/>
       </c>
       <c r="K5" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="6">
@@ -584,7 +597,7 @@
         <v/>
       </c>
       <c r="K6" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="7">
@@ -616,7 +629,7 @@
         <v/>
       </c>
       <c r="K7" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="8">
@@ -648,7 +661,7 @@
         <v/>
       </c>
       <c r="K8" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="9">
@@ -680,7 +693,7 @@
         <v/>
       </c>
       <c r="K9" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="10">
@@ -712,7 +725,7 @@
         <v/>
       </c>
       <c r="K10" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="11">
@@ -744,7 +757,7 @@
         <v/>
       </c>
       <c r="K11" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="12">
@@ -776,7 +789,7 @@
         <v/>
       </c>
       <c r="K12" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="13">
@@ -808,7 +821,7 @@
         <v/>
       </c>
       <c r="K13" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="14">
@@ -840,7 +853,7 @@
         <v/>
       </c>
       <c r="K14" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="15">
@@ -872,7 +885,7 @@
         <v/>
       </c>
       <c r="K15" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="16">
@@ -904,7 +917,7 @@
         <v/>
       </c>
       <c r="K16" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="17">
@@ -936,7 +949,7 @@
         <v/>
       </c>
       <c r="K17" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="18">
@@ -968,7 +981,7 @@
         <v/>
       </c>
       <c r="K18" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="19">
@@ -1000,7 +1013,7 @@
         <v/>
       </c>
       <c r="K19" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="20">
@@ -1032,7 +1045,7 @@
         <v/>
       </c>
       <c r="K20" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="21">
@@ -1064,7 +1077,7 @@
         <v/>
       </c>
       <c r="K21" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="22">
@@ -1096,7 +1109,7 @@
         <v/>
       </c>
       <c r="K22" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="23">
@@ -1128,7 +1141,7 @@
         <v/>
       </c>
       <c r="K23" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="24">
@@ -1160,7 +1173,7 @@
         <v/>
       </c>
       <c r="K24" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="25">
@@ -1192,7 +1205,7 @@
         <v/>
       </c>
       <c r="K25" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="26">
@@ -1224,7 +1237,7 @@
         <v/>
       </c>
       <c r="K26" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="27">
@@ -1256,7 +1269,7 @@
         <v/>
       </c>
       <c r="K27" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="28">
@@ -1288,7 +1301,7 @@
         <v/>
       </c>
       <c r="K28" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="29">
@@ -1320,7 +1333,7 @@
         <v/>
       </c>
       <c r="K29" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="30">
@@ -1352,7 +1365,7 @@
         <v/>
       </c>
       <c r="K30" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="31">
@@ -1384,7 +1397,7 @@
         <v/>
       </c>
       <c r="K31" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="32">
@@ -1416,7 +1429,7 @@
         <v/>
       </c>
       <c r="K32" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="33">
@@ -1448,7 +1461,7 @@
         <v/>
       </c>
       <c r="K33" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="34">
@@ -1480,7 +1493,7 @@
         <v/>
       </c>
       <c r="K34" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="35">
@@ -1512,7 +1525,7 @@
         <v/>
       </c>
       <c r="K35" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="36">
@@ -1544,7 +1557,7 @@
         <v/>
       </c>
       <c r="K36" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="37">
@@ -1576,7 +1589,7 @@
         <v/>
       </c>
       <c r="K37" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="38">
@@ -1608,7 +1621,7 @@
         <v/>
       </c>
       <c r="K38" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="39">
@@ -1640,7 +1653,7 @@
         <v/>
       </c>
       <c r="K39" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="40">
@@ -1672,7 +1685,7 @@
         <v/>
       </c>
       <c r="K40" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="41">
@@ -1704,7 +1717,7 @@
         <v/>
       </c>
       <c r="K41" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="42">
@@ -1736,7 +1749,7 @@
         <v/>
       </c>
       <c r="K42" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="43">
@@ -1768,7 +1781,7 @@
         <v/>
       </c>
       <c r="K43" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="44">
@@ -1800,7 +1813,7 @@
         <v/>
       </c>
       <c r="K44" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="45">
@@ -1832,7 +1845,7 @@
         <v/>
       </c>
       <c r="K45" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="46">
@@ -1864,7 +1877,7 @@
         <v/>
       </c>
       <c r="K46" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="47">
@@ -1896,7 +1909,7 @@
         <v/>
       </c>
       <c r="K47" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="48">
@@ -1928,7 +1941,7 @@
         <v/>
       </c>
       <c r="K48" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="49">
@@ -1960,7 +1973,7 @@
         <v/>
       </c>
       <c r="K49" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="50">
@@ -1992,7 +2005,7 @@
         <v/>
       </c>
       <c r="K50" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="51">
@@ -2024,7 +2037,7 @@
         <v/>
       </c>
       <c r="K51" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="52">
@@ -2056,7 +2069,7 @@
         <v/>
       </c>
       <c r="K52" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="53">
@@ -2088,7 +2101,7 @@
         <v/>
       </c>
       <c r="K53" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="54">
@@ -2120,7 +2133,7 @@
         <v/>
       </c>
       <c r="K54" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="55">
@@ -2152,7 +2165,7 @@
         <v/>
       </c>
       <c r="K55" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="56">
@@ -2184,7 +2197,7 @@
         <v/>
       </c>
       <c r="K56" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="57">
@@ -2216,7 +2229,7 @@
         <v/>
       </c>
       <c r="K57" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="58">
@@ -2248,7 +2261,7 @@
         <v/>
       </c>
       <c r="K58" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="59">
@@ -2280,7 +2293,7 @@
         <v/>
       </c>
       <c r="K59" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="60">
@@ -2312,7 +2325,7 @@
         <v/>
       </c>
       <c r="K60" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="61">
@@ -2344,7 +2357,7 @@
         <v/>
       </c>
       <c r="K61" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="62">
@@ -2376,7 +2389,7 @@
         <v/>
       </c>
       <c r="K62" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="63">
@@ -2408,7 +2421,7 @@
         <v/>
       </c>
       <c r="K63" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="64">
@@ -2440,7 +2453,7 @@
         <v/>
       </c>
       <c r="K64" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="65">
@@ -2472,7 +2485,7 @@
         <v/>
       </c>
       <c r="K65" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="66">
@@ -2504,7 +2517,7 @@
         <v/>
       </c>
       <c r="K66" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="67">
@@ -2536,7 +2549,7 @@
         <v/>
       </c>
       <c r="K67" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="68">
@@ -2568,7 +2581,7 @@
         <v/>
       </c>
       <c r="K68" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="69">
@@ -2600,7 +2613,7 @@
         <v/>
       </c>
       <c r="K69" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="70">
@@ -2632,7 +2645,7 @@
         <v/>
       </c>
       <c r="K70" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="71">
@@ -2664,7 +2677,7 @@
         <v/>
       </c>
       <c r="K71" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="72">
@@ -2696,7 +2709,7 @@
         <v/>
       </c>
       <c r="K72" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="73">
@@ -2728,7 +2741,7 @@
         <v/>
       </c>
       <c r="K73" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="74">
@@ -2760,7 +2773,7 @@
         <v/>
       </c>
       <c r="K74" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="75">
@@ -2792,7 +2805,7 @@
         <v/>
       </c>
       <c r="K75" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="76">
@@ -2824,7 +2837,7 @@
         <v/>
       </c>
       <c r="K76" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="77">
@@ -2856,7 +2869,7 @@
         <v/>
       </c>
       <c r="K77" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="78">
@@ -2888,7 +2901,7 @@
         <v/>
       </c>
       <c r="K78" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="79">
@@ -2920,7 +2933,7 @@
         <v/>
       </c>
       <c r="K79" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="80">
@@ -2952,7 +2965,7 @@
         <v/>
       </c>
       <c r="K80" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="81">
@@ -2984,7 +2997,7 @@
         <v/>
       </c>
       <c r="K81" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="82">
@@ -3016,7 +3029,7 @@
         <v/>
       </c>
       <c r="K82" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="83">
@@ -3048,7 +3061,7 @@
         <v/>
       </c>
       <c r="K83" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="84">
@@ -3080,7 +3093,7 @@
         <v/>
       </c>
       <c r="K84" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="85">
@@ -3112,7 +3125,7 @@
         <v/>
       </c>
       <c r="K85" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="86">
@@ -3144,7 +3157,7 @@
         <v/>
       </c>
       <c r="K86" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="87">
@@ -3176,7 +3189,7 @@
         <v/>
       </c>
       <c r="K87" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="88">
@@ -3208,7 +3221,7 @@
         <v/>
       </c>
       <c r="K88" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="89">
@@ -3240,7 +3253,7 @@
         <v/>
       </c>
       <c r="K89" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="90">
@@ -3272,7 +3285,7 @@
         <v/>
       </c>
       <c r="K90" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="91">
@@ -3304,7 +3317,7 @@
         <v/>
       </c>
       <c r="K91" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="92">
@@ -3336,7 +3349,7 @@
         <v/>
       </c>
       <c r="K92" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="93">
@@ -3368,7 +3381,7 @@
         <v/>
       </c>
       <c r="K93" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="94">
@@ -3400,7 +3413,7 @@
         <v/>
       </c>
       <c r="K94" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="95">
@@ -3432,7 +3445,7 @@
         <v/>
       </c>
       <c r="K95" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="96">
@@ -3464,7 +3477,7 @@
         <v/>
       </c>
       <c r="K96" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="97">
@@ -3496,7 +3509,7 @@
         <v/>
       </c>
       <c r="K97" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="98">
@@ -3528,7 +3541,7 @@
         <v/>
       </c>
       <c r="K98" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="99">
@@ -3560,7 +3573,7 @@
         <v/>
       </c>
       <c r="K99" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="100">
@@ -3592,7 +3605,7 @@
         <v/>
       </c>
       <c r="K100" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="101">
@@ -3624,7 +3637,7 @@
         <v/>
       </c>
       <c r="K101" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="102">
@@ -3656,7 +3669,7 @@
         <v/>
       </c>
       <c r="K102" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="103">
@@ -3688,7 +3701,7 @@
         <v/>
       </c>
       <c r="K103" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="104">
@@ -3720,7 +3733,7 @@
         <v/>
       </c>
       <c r="K104" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="105">
@@ -3752,7 +3765,7 @@
         <v/>
       </c>
       <c r="K105" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="106">
@@ -3784,7 +3797,7 @@
         <v/>
       </c>
       <c r="K106" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="107">
@@ -3816,7 +3829,7 @@
         <v/>
       </c>
       <c r="K107" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="108">
@@ -3848,7 +3861,7 @@
         <v/>
       </c>
       <c r="K108" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="109">
@@ -3880,7 +3893,7 @@
         <v/>
       </c>
       <c r="K109" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="110">
@@ -3912,7 +3925,7 @@
         <v/>
       </c>
       <c r="K110" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="111">
@@ -3944,7 +3957,7 @@
         <v/>
       </c>
       <c r="K111" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="112">
@@ -3976,7 +3989,7 @@
         <v/>
       </c>
       <c r="K112" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="113">
@@ -4008,7 +4021,7 @@
         <v/>
       </c>
       <c r="K113" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="114">
@@ -4040,7 +4053,7 @@
         <v/>
       </c>
       <c r="K114" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="115">
@@ -4072,7 +4085,7 @@
         <v/>
       </c>
       <c r="K115" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="116">
@@ -4104,7 +4117,7 @@
         <v/>
       </c>
       <c r="K116" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="117">
@@ -4136,7 +4149,7 @@
         <v/>
       </c>
       <c r="K117" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="118">
@@ -4168,7 +4181,7 @@
         <v/>
       </c>
       <c r="K118" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="119">
@@ -4200,7 +4213,7 @@
         <v/>
       </c>
       <c r="K119" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="120">
@@ -4232,7 +4245,7 @@
         <v/>
       </c>
       <c r="K120" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="121">
@@ -4264,7 +4277,7 @@
         <v/>
       </c>
       <c r="K121" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="122">
@@ -4296,7 +4309,7 @@
         <v/>
       </c>
       <c r="K122" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="123">
@@ -4328,7 +4341,7 @@
         <v/>
       </c>
       <c r="K123" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="124">
@@ -4360,7 +4373,7 @@
         <v/>
       </c>
       <c r="K124" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="125">
@@ -4392,7 +4405,7 @@
         <v/>
       </c>
       <c r="K125" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="126">
@@ -4424,7 +4437,7 @@
         <v/>
       </c>
       <c r="K126" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="127">
@@ -4456,7 +4469,7 @@
         <v/>
       </c>
       <c r="K127" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="128">
@@ -4488,7 +4501,7 @@
         <v/>
       </c>
       <c r="K128" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="129">
@@ -4520,7 +4533,7 @@
         <v/>
       </c>
       <c r="K129" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="130">
@@ -4552,7 +4565,7 @@
         <v/>
       </c>
       <c r="K130" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="131">
@@ -4584,7 +4597,7 @@
         <v/>
       </c>
       <c r="K131" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="132">
@@ -4616,7 +4629,7 @@
         <v/>
       </c>
       <c r="K132" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="133">
@@ -4648,7 +4661,7 @@
         <v/>
       </c>
       <c r="K133" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="134">
@@ -4680,7 +4693,7 @@
         <v/>
       </c>
       <c r="K134" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="135">
@@ -4712,7 +4725,7 @@
         <v/>
       </c>
       <c r="K135" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="136">
@@ -4744,7 +4757,7 @@
         <v/>
       </c>
       <c r="K136" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="137">
@@ -4776,7 +4789,7 @@
         <v/>
       </c>
       <c r="K137" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="138">
@@ -4808,7 +4821,7 @@
         <v/>
       </c>
       <c r="K138" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="139">
@@ -4840,7 +4853,7 @@
         <v/>
       </c>
       <c r="K139" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="140">
@@ -4872,7 +4885,7 @@
         <v/>
       </c>
       <c r="K140" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="141">
@@ -4904,7 +4917,7 @@
         <v/>
       </c>
       <c r="K141" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="142">
@@ -4936,7 +4949,7 @@
         <v/>
       </c>
       <c r="K142" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="143">
@@ -4968,7 +4981,7 @@
         <v/>
       </c>
       <c r="K143" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="144">
@@ -5000,7 +5013,7 @@
         <v/>
       </c>
       <c r="K144" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="145">
@@ -5032,7 +5045,7 @@
         <v/>
       </c>
       <c r="K145" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="146">
@@ -5064,7 +5077,7 @@
         <v/>
       </c>
       <c r="K146" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="147">
@@ -5096,7 +5109,7 @@
         <v/>
       </c>
       <c r="K147" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="148">
@@ -5128,7 +5141,7 @@
         <v/>
       </c>
       <c r="K148" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="149">
@@ -5160,7 +5173,7 @@
         <v/>
       </c>
       <c r="K149" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
     <row r="150">
@@ -5192,7 +5205,7 @@
         <v/>
       </c>
       <c r="K150" t="str">
-        <v>MATERIALES</v>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>